<commit_message>
Working on scripts for doing model replacement
</commit_message>
<xml_diff>
--- a/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
+++ b/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubRepos\ApsimX\Prototypes\WheatSimpleLeaf\SimpleLeafImplementation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF67CA3D-17CD-4C3D-9190-CEC4A98F4B0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDED6FC4-781D-4268-8E17-0ACBC3371ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2295" yWindow="540" windowWidth="19455" windowHeight="12105" xr2:uid="{99730FEE-4914-42B9-ACDB-525A29E01521}"/>
+    <workbookView xWindow="-16320" yWindow="-5925" windowWidth="16440" windowHeight="28320" xr2:uid="{99730FEE-4914-42B9-ACDB-525A29E01521}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,91 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
-  <si>
-    <t>[Wheat].Grain.Nconc</t>
-  </si>
-  <si>
-    <t>[Wheat].Grain.NConc</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.MainStemPopulation</t>
-  </si>
-  <si>
-    <t>[Wheat].Population</t>
-  </si>
-  <si>
-    <t>sum([Soil].NO3.kgha)</t>
-  </si>
-  <si>
-    <t>sum([Soil].Water.MM)</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.CoverGreen</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.Canopy.CoverGreen</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.CoverTotal</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.Canopy.CoverTotal</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.Fn</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.FN</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.Fw</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.Canopy.FW</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.Height</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.Canopy.Height</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.LAI</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.Canopy.LAI</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.SpecificAreaCanopy</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.Canopy.SpecificArea</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.Transpiration</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.Canopy.Transpiration</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.StemNumberPerPlant</t>
-  </si>
-  <si>
-    <t>[Wheat].StemNumber</t>
-  </si>
-  <si>
-    <t>[Wheat].Leaf.StemPopulation</t>
-  </si>
-  <si>
-    <t>[Wheat].StemPopulation</t>
-  </si>
-  <si>
-    <t>[Wheat].Root.Depth</t>
-  </si>
-  <si>
-    <t>[Wheat].Root.Network.Depth</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="130">
   <si>
     <t>CohortLeaf</t>
   </si>
@@ -128,10 +44,388 @@
     <t>SimpleLeaf</t>
   </si>
   <si>
-    <t>sum([Soil].Water.MM) as ProfileWater</t>
-  </si>
-  <si>
-    <t>sum([Soil].NO3.kgha) as TotalNO3</t>
+    <t>[Phenology].Phyllochron.BasePhyllochron</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Tips</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.SpecificArea</t>
+  </si>
+  <si>
+    <t>Wheat.Phenology.HaunStage</t>
+  </si>
+  <si>
+    <t>Wheat.Phenology.PTQ</t>
+  </si>
+  <si>
+    <t>Wheat.Phenology.Phyllochron</t>
+  </si>
+  <si>
+    <t>Wheat.Arbitrator.DM.TotalFixationSupply</t>
+  </si>
+  <si>
+    <t>Wheat.Arbitrator.DM.TotalPlantDemand</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Live.StructuralWt</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Total.StructuralWt</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Live.StructuralN</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Total.StructuralN</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.MinimumNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.CriticalNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.MaximumNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.DMDemand.Total</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Live.StructuralWt</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Total.StructuralWt</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Live.StructuralN</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Total.StructuralN</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.MinimumNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.CriticalNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.MaximumNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.DMDemand.Total</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Live.StructuralWt</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Total.StructuralWt</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Live.StructuralN</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Total.StructuralN</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.DMDemand.Total</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.DMDemand.Total</t>
+  </si>
+  <si>
+    <t>Wheat.Root.DMDemand.Total</t>
+  </si>
+  <si>
+    <t>[Leaf].Phyllochron.BasePhyllochron</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.MainStemPopulation</t>
+  </si>
+  <si>
+    <t>Wheat.Population</t>
+  </si>
+  <si>
+    <t>sum(Soil.Water.MM)</t>
+  </si>
+  <si>
+    <t>sum(Soil.Water.MM) as ProfileWater</t>
+  </si>
+  <si>
+    <t>sum(Soil.NO3.kgha)</t>
+  </si>
+  <si>
+    <t>sum(Soil.NO3.kgha) as TotalNO3</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Nconc</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.NConc</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.CoverGreen</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Canopy.CoverGreen</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.CoverTotal</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Canopy.CoverTotal</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Fn</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.FN</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Fw</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Canopy.FW</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Height</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Canopy.Height</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.LAI</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Canopy.LAI</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.SpecificAreaCanopy</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Canopy.SpecificArea</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Transpiration</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Canopy.Transpiration</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.StemNumberPerPlant</t>
+  </si>
+  <si>
+    <t>Wheat.StemNumber</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.StemPopulation</t>
+  </si>
+  <si>
+    <t>Wheat.StemPopulation</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Depth</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Network.Depth</t>
+  </si>
+  <si>
+    <t>[Grain].NumberFunction.GrainNumber.GrainsPerGramOfStem</t>
+  </si>
+  <si>
+    <t>[Phenology].PhyllochronPpSensitivity</t>
+  </si>
+  <si>
+    <t>[Leaf].Canopy.GreenExtinctionCoefficient</t>
+  </si>
+  <si>
+    <t>[Leaf].PhyllochronPpSensitivity</t>
+  </si>
+  <si>
+    <t>[Grain].Number.GrainNumber.GrainsPerGramOfStem</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.HaunStage</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Phyllochron</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.MinimumNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.CriticalNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.MaximumNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Arbitrator.Carbon.TotalFixationSupply</t>
+  </si>
+  <si>
+    <t>Wheat.Arbitrator.Carbon.TotalPlantDemand</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Live.Wt.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Live.N.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Total.Wt.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Total.N.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Nitrogen.Concentration.Minimum</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Nitrogen.Concentration.Critical</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Nitrogen.Concentration.Maximum</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Carbon.Demands.Total</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Live.Wt.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Total.Wt.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Live.N.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Total.N.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Nitrogen.Concentration.Minimum</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Nitrogen.Concentration.Critical</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Nitrogen.Concentration.Maximum</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Carbon.Demands.Total</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Live.Wt.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Total.Wt.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Live.N.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Total.N.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Nitrogen.Concentration.Minimum</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Nitrogen.Concentration.Critical</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Nitrogen.Concentration.Maximum</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Carbon.Demands.Total</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Live.StructuralWt</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Live.Wt.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Total.StructuralWt</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Total.Wt.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Live.StructuralN</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Live.N.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Total.StructuralN</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Total.N.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.MinimumNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Nitrogen.Concentration.Minimum</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.CriticalNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Nitrogen.Concentration.Critical</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.MaximumNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Nitrogen.Concentration.Maximum</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Carbon.Demands.Total</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Live.StructuralWt</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Live.Wt.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Total.StructuralWt</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Total.Wt.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Live.StructuralN</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Live.N.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Total.StructuralN</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Total.N.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Root.MinimumNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Nitrogen.Concentration.Minimum</t>
+  </si>
+  <si>
+    <t>Wheat.Root.CriticalNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Nitrogen.Concentration.Critical</t>
+  </si>
+  <si>
+    <t>Wheat.Root.MaximumNConc</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Nitrogen.Concentration.Maximum</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Carbon.Demands.Total</t>
   </si>
 </sst>
 </file>
@@ -503,139 +797,544 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45DFA9DE-B569-4853-98A7-0B05A40C5DD2}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="57.140625" customWidth="1"/>
+    <col min="1" max="1" width="56.140625" customWidth="1"/>
     <col min="2" max="2" width="87.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s">
-        <v>1</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="B14" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>11</v>
+      </c>
+      <c r="B29" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>15</v>
+      </c>
+      <c r="B33" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>16</v>
+      </c>
+      <c r="B34" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>17</v>
+      </c>
+      <c r="B35" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>18</v>
+      </c>
+      <c r="B36" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>19</v>
+      </c>
+      <c r="B37" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>20</v>
+      </c>
+      <c r="B38" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>21</v>
+      </c>
+      <c r="B39" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>22</v>
+      </c>
+      <c r="B40" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>23</v>
+      </c>
+      <c r="B41" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>24</v>
+      </c>
+      <c r="B42" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>25</v>
+      </c>
+      <c r="B43" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>26</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B44" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>27</v>
+      </c>
+      <c r="B45" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>28</v>
+      </c>
+      <c r="B46" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>29</v>
+      </c>
+      <c r="B47" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>71</v>
+      </c>
+      <c r="B48" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>72</v>
+      </c>
+      <c r="B49" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>73</v>
+      </c>
+      <c r="B50" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>30</v>
+      </c>
+      <c r="B51" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>100</v>
+      </c>
+      <c r="B52" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>102</v>
+      </c>
+      <c r="B53" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>104</v>
+      </c>
+      <c r="B54" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>106</v>
+      </c>
+      <c r="B55" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>108</v>
+      </c>
+      <c r="B56" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>110</v>
+      </c>
+      <c r="B57" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>112</v>
+      </c>
+      <c r="B58" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>31</v>
+      </c>
+      <c r="B59" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>115</v>
+      </c>
+      <c r="B60" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>117</v>
+      </c>
+      <c r="B61" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>119</v>
+      </c>
+      <c r="B62" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>121</v>
+      </c>
+      <c r="B63" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>123</v>
+      </c>
+      <c r="B64" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>125</v>
+      </c>
+      <c r="B65" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>127</v>
+      </c>
+      <c r="B66" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>32</v>
+      </c>
+      <c r="B67" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Scripts to introduce new wheat model
</commit_message>
<xml_diff>
--- a/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
+++ b/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubRepos\ApsimX\Prototypes\WheatSimpleLeaf\SimpleLeafImplementation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDED6FC4-781D-4268-8E17-0ACBC3371ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A6EB82D-3F87-4907-8E03-778612BDF80F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-16320" yWindow="-5925" windowWidth="16440" windowHeight="28320" xr2:uid="{99730FEE-4914-42B9-ACDB-525A29E01521}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="135">
   <si>
     <t>CohortLeaf</t>
   </si>
@@ -266,18 +266,6 @@
     <t>Wheat.Arbitrator.Carbon.TotalPlantDemand</t>
   </si>
   <si>
-    <t>Wheat.Stem.Live.Wt.Structural</t>
-  </si>
-  <si>
-    <t>Wheat.Stem.Live.N.Structural</t>
-  </si>
-  <si>
-    <t>Wheat.Stem.Total.Wt.Structural</t>
-  </si>
-  <si>
-    <t>Wheat.Stem.Total.N.Structural</t>
-  </si>
-  <si>
     <t>Wheat.Stem.Nitrogen.Concentration.Minimum</t>
   </si>
   <si>
@@ -290,18 +278,6 @@
     <t>Wheat.Stem.Carbon.Demands.Total</t>
   </si>
   <si>
-    <t>Wheat.Spike.Live.Wt.Structural</t>
-  </si>
-  <si>
-    <t>Wheat.Spike.Total.Wt.Structural</t>
-  </si>
-  <si>
-    <t>Wheat.Spike.Live.N.Structural</t>
-  </si>
-  <si>
-    <t>Wheat.Spike.Total.N.Structural</t>
-  </si>
-  <si>
     <t>Wheat.Spike.Nitrogen.Concentration.Minimum</t>
   </si>
   <si>
@@ -314,18 +290,6 @@
     <t>Wheat.Spike.Carbon.Demands.Total</t>
   </si>
   <si>
-    <t>Wheat.Leaf.Live.Wt.Structural</t>
-  </si>
-  <si>
-    <t>Wheat.Leaf.Total.Wt.Structural</t>
-  </si>
-  <si>
-    <t>Wheat.Leaf.Live.N.Structural</t>
-  </si>
-  <si>
-    <t>Wheat.Leaf.Total.N.Structural</t>
-  </si>
-  <si>
     <t>Wheat.Leaf.Nitrogen.Concentration.Minimum</t>
   </si>
   <si>
@@ -341,27 +305,15 @@
     <t>Wheat.Grain.Live.StructuralWt</t>
   </si>
   <si>
-    <t>Wheat.Grain.Live.Wt.Structural</t>
-  </si>
-  <si>
     <t>Wheat.Grain.Total.StructuralWt</t>
   </si>
   <si>
-    <t>Wheat.Grain.Total.Wt.Structural</t>
-  </si>
-  <si>
     <t>Wheat.Grain.Live.StructuralN</t>
   </si>
   <si>
-    <t>Wheat.Grain.Live.N.Structural</t>
-  </si>
-  <si>
     <t>Wheat.Grain.Total.StructuralN</t>
   </si>
   <si>
-    <t>Wheat.Grain.Total.N.Structural</t>
-  </si>
-  <si>
     <t>Wheat.Grain.MinimumNConc</t>
   </si>
   <si>
@@ -386,27 +338,15 @@
     <t>Wheat.Root.Live.StructuralWt</t>
   </si>
   <si>
-    <t>Wheat.Root.Live.Wt.Structural</t>
-  </si>
-  <si>
     <t>Wheat.Root.Total.StructuralWt</t>
   </si>
   <si>
-    <t>Wheat.Root.Total.Wt.Structural</t>
-  </si>
-  <si>
     <t>Wheat.Root.Live.StructuralN</t>
   </si>
   <si>
-    <t>Wheat.Root.Live.N.Structural</t>
-  </si>
-  <si>
     <t>Wheat.Root.Total.StructuralN</t>
   </si>
   <si>
-    <t>Wheat.Root.Total.N.Structural</t>
-  </si>
-  <si>
     <t>Wheat.Root.MinimumNConc</t>
   </si>
   <si>
@@ -426,6 +366,81 @@
   </si>
   <si>
     <t>Wheat.Root.Carbon.Demands.Total</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.SpecificNitrogen</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Canopy.SpecificNitrogen</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Total.Weight.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Live.Weight.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Live.Weight.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Total.Weight.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Live.Weight.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Total.Weight.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Live.Weight.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Total.Weight.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Live.Weight.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Total.Weight.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Live.Nitrogen.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.Total.Nitrogen.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Live.Nitrogen.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Grain.Total.Nitrogen.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Live.Nitrogen.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Total.Nitrogen.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Live.Nitrogen.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Stem.Total.Nitrogen.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Live.Nitrogen.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Spike.Total.Nitrogen.Structural</t>
+  </si>
+  <si>
+    <t>Wheat.Root.WaterUptake</t>
+  </si>
+  <si>
+    <t>Wheat.Root.Network.WaterUptake</t>
+  </si>
+  <si>
+    <t>Wheat.Structure.TotalStemPopn</t>
   </si>
 </sst>
 </file>
@@ -797,7 +812,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45DFA9DE-B569-4853-98A7-0B05A40C5DD2}">
-  <dimension ref="A1:B67"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.140625" customWidth="1"/>
@@ -934,407 +949,434 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>110</v>
       </c>
       <c r="B17" t="s">
-        <v>57</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B18" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B19" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B20" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>3</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="B24" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B26" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>78</v>
+        <v>113</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B30" t="s">
-        <v>77</v>
+        <v>112</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B31" t="s">
-        <v>79</v>
+        <v>128</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B32" t="s">
-        <v>80</v>
+        <v>129</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B33" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B34" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B35" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B36" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B37" t="s">
-        <v>85</v>
+        <v>114</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B38" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B39" t="s">
-        <v>87</v>
+        <v>130</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B40" t="s">
-        <v>88</v>
+        <v>131</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B41" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B43" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B44" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B45" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B46" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B47" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="B48" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B49" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B50" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>30</v>
+        <v>73</v>
       </c>
       <c r="B51" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="B52" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="B53" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="B54" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="B55" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="B56" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="B57" t="s">
-        <v>111</v>
+        <v>93</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="B58" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>31</v>
+        <v>96</v>
       </c>
       <c r="B59" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>115</v>
+        <v>31</v>
       </c>
       <c r="B60" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="B61" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>119</v>
+        <v>100</v>
       </c>
       <c r="B62" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="B63" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>123</v>
+        <v>102</v>
       </c>
       <c r="B64" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="B65" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="B66" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>107</v>
+      </c>
+      <c r="B67" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
         <v>32</v>
       </c>
-      <c r="B67" t="s">
-        <v>129</v>
+      <c r="B68" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>132</v>
+      </c>
+      <c r="B69" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>134</v>
+      </c>
+      <c r="B70" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finalising scripts to introduce new model into test set
</commit_message>
<xml_diff>
--- a/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
+++ b/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubRepos\ApsimX\Prototypes\WheatSimpleLeaf\SimpleLeafImplementation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C01C7D0-D075-48ED-9154-865740865C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA3BFE68-6CC6-46CE-84CF-FF8A37335B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{99730FEE-4914-42B9-ACDB-525A29E01521}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{99730FEE-4914-42B9-ACDB-525A29E01521}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="SimpleLeafRenames" sheetId="1" r:id="rId1"/>
     <sheet name="Existing Model renames" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
   </sheets>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="187">
   <si>
     <t>CohortLeaf</t>
   </si>
@@ -624,12 +624,18 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -659,12 +665,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1001,11 +1011,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45DFA9DE-B569-4853-98A7-0B05A40C5DD2}">
-  <dimension ref="A1:B90"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:B100"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="56.140625" customWidth="1"/>
-    <col min="2" max="2" width="87.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="56.109375" customWidth="1"/>
+    <col min="2" max="2" width="87.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1017,714 +1027,794 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
-        <v>72</v>
+      <c r="A2" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>73</v>
+      <c r="A3" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B4" t="s">
-        <v>93</v>
+      <c r="A4" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" t="s">
-        <v>96</v>
+      <c r="A5" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B6" t="s">
-        <v>122</v>
+      <c r="A6" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="B7" t="s">
-        <v>116</v>
+      <c r="A7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="B8" t="s">
-        <v>95</v>
+      <c r="A8" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B9" t="s">
-        <v>91</v>
+      <c r="A9" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B10" t="s">
-        <v>153</v>
+      <c r="A10" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="B11" t="s">
-        <v>154</v>
+      <c r="A11" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>38</v>
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
-        <v>89</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>123</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B14" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="B17" t="s">
-        <v>83</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1" t="s">
-        <v>30</v>
+        <v>94</v>
       </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>156</v>
+        <v>90</v>
+      </c>
+      <c r="B19" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1" t="s">
-        <v>44</v>
+        <v>133</v>
       </c>
       <c r="B20" t="s">
-        <v>45</v>
+        <v>153</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1" t="s">
-        <v>46</v>
+        <v>134</v>
       </c>
       <c r="B21" t="s">
-        <v>47</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B22" t="s">
-        <v>49</v>
+        <v>39</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1" t="s">
-        <v>136</v>
+        <v>89</v>
       </c>
       <c r="B23" t="s">
-        <v>157</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="1" t="s">
-        <v>137</v>
+        <v>87</v>
       </c>
       <c r="B24" t="s">
-        <v>158</v>
+        <v>117</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="1" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>138</v>
+        <v>42</v>
       </c>
       <c r="B26" t="s">
-        <v>159</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>140</v>
+        <v>70</v>
+      </c>
+      <c r="B27" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>120</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B29" t="s">
-        <v>114</v>
+        <v>135</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B30" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="1" t="s">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="B31" t="s">
-        <v>84</v>
+        <v>47</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="1" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="B32" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="1" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B33" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="1" t="s">
-        <v>4</v>
+        <v>137</v>
       </c>
       <c r="B34" t="s">
-        <v>53</v>
+        <v>158</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B35" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="1" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B36" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B37" t="s">
-        <v>109</v>
+        <v>139</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="1" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="B38" t="s">
-        <v>57</v>
+        <v>120</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="B39" t="s">
-        <v>59</v>
+        <v>114</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="1" t="s">
-        <v>143</v>
+        <v>34</v>
       </c>
       <c r="B40" t="s">
-        <v>162</v>
+        <v>35</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>3</v>
+        <v>71</v>
       </c>
       <c r="B41" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="B42" t="s">
-        <v>121</v>
+        <v>82</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="1" t="s">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B43" t="s">
-        <v>115</v>
+        <v>160</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="1" t="s">
-        <v>54</v>
+        <v>4</v>
       </c>
       <c r="B44" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="1" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="B45" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B46" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>145</v>
+        <v>108</v>
       </c>
       <c r="B47" t="s">
-        <v>164</v>
+        <v>109</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="1" t="s">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="B48" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="1" t="s">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="B49" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="1" t="s">
-        <v>103</v>
+        <v>143</v>
       </c>
       <c r="B50" t="s">
-        <v>104</v>
+        <v>162</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="1" t="s">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="B51" t="s">
-        <v>107</v>
+        <v>67</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="1" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="B52" t="s">
-        <v>61</v>
+        <v>121</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>99</v>
+        <v>27</v>
       </c>
       <c r="B53" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="1" t="s">
-        <v>97</v>
+        <v>54</v>
       </c>
       <c r="B54" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="1" t="s">
-        <v>105</v>
+        <v>5</v>
       </c>
       <c r="B55" t="s">
-        <v>106</v>
+        <v>67</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="1" t="s">
-        <v>101</v>
+        <v>144</v>
       </c>
       <c r="B56" t="s">
-        <v>102</v>
+        <v>163</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="1" t="s">
-        <v>100</v>
+        <v>145</v>
       </c>
       <c r="B57" t="s">
-        <v>125</v>
+        <v>164</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="1" t="s">
-        <v>98</v>
+        <v>6</v>
       </c>
       <c r="B58" t="s">
-        <v>119</v>
+        <v>67</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="1" t="s">
-        <v>130</v>
+        <v>7</v>
       </c>
       <c r="B59" t="s">
-        <v>131</v>
+        <v>68</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="1" t="s">
-        <v>23</v>
+        <v>103</v>
       </c>
       <c r="B60" t="s">
-        <v>79</v>
+        <v>104</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="1" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B61" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="1" t="s">
-        <v>146</v>
+        <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>165</v>
+        <v>61</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="1" t="s">
-        <v>147</v>
+        <v>99</v>
       </c>
       <c r="B63" t="s">
-        <v>166</v>
+        <v>124</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="1" t="s">
-        <v>148</v>
+        <v>97</v>
       </c>
       <c r="B64" t="s">
-        <v>167</v>
+        <v>118</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="1" t="s">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="B65" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="1" t="s">
-        <v>18</v>
+        <v>101</v>
       </c>
       <c r="B66" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="1" t="s">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="B67" t="s">
-        <v>80</v>
+        <v>125</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="1" t="s">
-        <v>22</v>
+        <v>98</v>
       </c>
       <c r="B68" t="s">
-        <v>78</v>
+        <v>119</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>168</v>
+        <v>130</v>
+      </c>
+      <c r="B69" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B70" t="s">
-        <v>129</v>
+        <v>79</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="1" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B71" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="1" t="s">
-        <v>15</v>
+        <v>146</v>
       </c>
       <c r="B72" t="s">
-        <v>75</v>
+        <v>165</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="1" t="s">
-        <v>17</v>
+        <v>147</v>
       </c>
       <c r="B73" t="s">
-        <v>77</v>
+        <v>166</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="1" t="s">
-        <v>12</v>
+        <v>148</v>
       </c>
       <c r="B74" t="s">
-        <v>126</v>
+        <v>167</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="1" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B75" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B76" t="s">
-        <v>76</v>
+        <v>112</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="1" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B77" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>169</v>
+        <v>22</v>
+      </c>
+      <c r="B78" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B79" t="s">
-        <v>127</v>
+        <v>149</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="1" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B80" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="1" t="s">
-        <v>151</v>
+        <v>19</v>
       </c>
       <c r="B81" t="s">
-        <v>170</v>
+        <v>113</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="1" t="s">
-        <v>132</v>
+        <v>15</v>
       </c>
       <c r="B82" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="1" t="s">
-        <v>152</v>
+        <v>17</v>
       </c>
       <c r="B83" t="s">
-        <v>171</v>
+        <v>77</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="1" t="s">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="B84" t="s">
-        <v>66</v>
+        <v>126</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="1" t="s">
-        <v>64</v>
+        <v>10</v>
       </c>
       <c r="B85" t="s">
-        <v>64</v>
+        <v>111</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="1" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="B86" t="s">
-        <v>33</v>
+        <v>76</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="1" t="s">
-        <v>63</v>
+        <v>14</v>
       </c>
       <c r="B87" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B89" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B90" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B91" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B92" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B93" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B94" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B95" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B96" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B97" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B98" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="89" spans="1:2">
-      <c r="A89" t="s">
+    <row r="99" spans="1:2">
+      <c r="A99" t="s">
         <v>172</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B99" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="90" spans="1:2">
-      <c r="A90" t="s">
+    <row r="100" spans="1:2">
+      <c r="A100" t="s">
         <v>173</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B100" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1736,10 +1826,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F34CFB7-6746-4EED-A01C-0BEF089865E6}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="42.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1838,7 +1928,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8C94458-8D2F-45A6-90CE-3561672AE312}">
   <dimension ref="A1:B89"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="79" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Fix wrong variable name replace
</commit_message>
<xml_diff>
--- a/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
+++ b/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubRepos\ApsimX\Prototypes\WheatSimpleLeaf\SimpleLeafImplementation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA3BFE68-6CC6-46CE-84CF-FF8A37335B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{743CED89-89BC-4A02-B161-5D885986D717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{99730FEE-4914-42B9-ACDB-525A29E01521}"/>
+    <workbookView xWindow="-16320" yWindow="-5925" windowWidth="16440" windowHeight="28320" xr2:uid="{99730FEE-4914-42B9-ACDB-525A29E01521}"/>
   </bookViews>
   <sheets>
     <sheet name="SimpleLeafRenames" sheetId="1" r:id="rId1"/>
@@ -1012,10 +1012,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45DFA9DE-B569-4853-98A7-0B05A40C5DD2}">
   <dimension ref="A1:B100"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="56.109375" customWidth="1"/>
-    <col min="2" max="2" width="87.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="56.140625" customWidth="1"/>
+    <col min="2" max="2" width="87.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1084,7 +1084,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="3" t="s">
-        <v>183</v>
+        <v>151</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>170</v>
@@ -1826,10 +1826,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F34CFB7-6746-4EED-A01C-0BEF089865E6}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="42.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="48.140625" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1928,7 +1928,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8C94458-8D2F-45A6-90CE-3561672AE312}">
   <dimension ref="A1:B89"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="79" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
setting up comparison graphs
</commit_message>
<xml_diff>
--- a/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
+++ b/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubRepos\ApsimX\Prototypes\WheatSimpleLeaf\SimpleLeafImplementation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD8FCC7-85A4-4F1D-B97F-B95BB6444D0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23FC5128-BD09-426B-8BE9-80AA61BCDE75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-5925" windowWidth="16440" windowHeight="28320" xr2:uid="{99730FEE-4914-42B9-ACDB-525A29E01521}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{99730FEE-4914-42B9-ACDB-525A29E01521}"/>
   </bookViews>
   <sheets>
     <sheet name="SimpleLeafRenames" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="192">
   <si>
     <t>CohortLeaf</t>
   </si>
@@ -1026,11 +1026,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45DFA9DE-B569-4853-98A7-0B05A40C5DD2}">
-  <dimension ref="A1:B104"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:B99"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="56.140625" customWidth="1"/>
-    <col min="2" max="2" width="87.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="56.109375" customWidth="1"/>
+    <col min="2" max="2" width="87.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1203,279 +1203,279 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>38</v>
+        <v>89</v>
+      </c>
+      <c r="B22" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B23" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="1" t="s">
-        <v>87</v>
+        <v>40</v>
       </c>
       <c r="B24" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B25" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="1" t="s">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="B26" t="s">
-        <v>43</v>
+        <v>83</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="1" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="B27" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="1" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="B28" t="s">
-        <v>85</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>156</v>
+        <v>46</v>
+      </c>
+      <c r="B29" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B30" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="1" t="s">
-        <v>46</v>
+        <v>136</v>
       </c>
       <c r="B31" t="s">
-        <v>47</v>
+        <v>157</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>137</v>
       </c>
       <c r="B32" t="s">
-        <v>49</v>
+        <v>158</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="1" t="s">
-        <v>136</v>
+        <v>50</v>
       </c>
       <c r="B33" t="s">
-        <v>157</v>
+        <v>51</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B34" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="1" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="B35" t="s">
-        <v>51</v>
+        <v>120</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="1" t="s">
-        <v>138</v>
+        <v>26</v>
       </c>
       <c r="B36" t="s">
-        <v>159</v>
+        <v>114</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>140</v>
+        <v>184</v>
+      </c>
+      <c r="B37" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="1" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>120</v>
+        <v>35</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
-        <v>26</v>
+        <v>71</v>
       </c>
       <c r="B39" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="1" t="s">
-        <v>184</v>
+        <v>69</v>
       </c>
       <c r="B40" t="s">
-        <v>185</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="B41" t="s">
-        <v>35</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>84</v>
+        <v>53</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="1" t="s">
-        <v>69</v>
+        <v>142</v>
       </c>
       <c r="B43" t="s">
-        <v>82</v>
+        <v>161</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="1" t="s">
-        <v>4</v>
+        <v>108</v>
       </c>
       <c r="B44" t="s">
-        <v>53</v>
+        <v>109</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B45" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="1" t="s">
-        <v>142</v>
+        <v>58</v>
       </c>
       <c r="B46" t="s">
-        <v>161</v>
+        <v>59</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>108</v>
+        <v>143</v>
       </c>
       <c r="B47" t="s">
-        <v>109</v>
+        <v>162</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="1" t="s">
-        <v>56</v>
+        <v>184</v>
       </c>
       <c r="B48" t="s">
-        <v>57</v>
+        <v>185</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="1" t="s">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="B49" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="1" t="s">
-        <v>143</v>
+        <v>29</v>
       </c>
       <c r="B50" t="s">
-        <v>162</v>
+        <v>121</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="1" t="s">
-        <v>184</v>
+        <v>27</v>
       </c>
       <c r="B51" t="s">
-        <v>185</v>
+        <v>115</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="1" t="s">
-        <v>3</v>
+        <v>54</v>
       </c>
       <c r="B52" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="B53" t="s">
-        <v>121</v>
+        <v>67</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="1" t="s">
-        <v>27</v>
+        <v>144</v>
       </c>
       <c r="B54" t="s">
-        <v>115</v>
+        <v>163</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="1" t="s">
-        <v>54</v>
+        <v>145</v>
       </c>
       <c r="B55" t="s">
-        <v>55</v>
+        <v>164</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B56" t="s">
         <v>67</v>
@@ -1483,385 +1483,345 @@
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="1" t="s">
-        <v>144</v>
+        <v>7</v>
       </c>
       <c r="B57" t="s">
-        <v>163</v>
+        <v>68</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="1" t="s">
-        <v>145</v>
+        <v>103</v>
       </c>
       <c r="B58" t="s">
-        <v>164</v>
+        <v>104</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="1" t="s">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="B59" t="s">
-        <v>67</v>
+        <v>107</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="1" t="s">
-        <v>7</v>
+        <v>60</v>
       </c>
       <c r="B60" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="1" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B61" t="s">
-        <v>104</v>
+        <v>124</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="1" t="s">
-        <v>32</v>
+        <v>97</v>
       </c>
       <c r="B62" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="1" t="s">
-        <v>60</v>
+        <v>105</v>
       </c>
       <c r="B63" t="s">
-        <v>61</v>
+        <v>106</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B64" t="s">
-        <v>124</v>
+        <v>102</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" s="1" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B65" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="1" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="B66" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" s="1" t="s">
-        <v>101</v>
+        <v>130</v>
       </c>
       <c r="B67" t="s">
-        <v>102</v>
+        <v>131</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" s="1" t="s">
-        <v>100</v>
+        <v>23</v>
       </c>
       <c r="B68" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" s="1" t="s">
-        <v>98</v>
+        <v>25</v>
       </c>
       <c r="B69" t="s">
-        <v>119</v>
+        <v>81</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" s="1" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
       <c r="B70" t="s">
-        <v>131</v>
+        <v>165</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71" s="1" t="s">
-        <v>23</v>
+        <v>147</v>
       </c>
       <c r="B71" t="s">
-        <v>79</v>
+        <v>166</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" s="1" t="s">
-        <v>25</v>
+        <v>148</v>
       </c>
       <c r="B72" t="s">
-        <v>81</v>
+        <v>167</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" s="1" t="s">
-        <v>146</v>
+        <v>20</v>
       </c>
       <c r="B73" t="s">
-        <v>165</v>
+        <v>128</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" s="1" t="s">
-        <v>147</v>
+        <v>18</v>
       </c>
       <c r="B74" t="s">
-        <v>166</v>
+        <v>112</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" s="1" t="s">
-        <v>148</v>
+        <v>24</v>
       </c>
       <c r="B75" t="s">
-        <v>167</v>
+        <v>80</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B76" t="s">
-        <v>128</v>
+        <v>78</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B77" t="s">
-        <v>112</v>
+        <v>186</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B78" t="s">
-        <v>80</v>
+        <v>129</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B79" t="s">
-        <v>78</v>
+        <v>113</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>168</v>
+        <v>15</v>
+      </c>
+      <c r="B80" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>188</v>
+        <v>17</v>
+      </c>
+      <c r="B81" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" s="1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="B82" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" s="1" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B83" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B84" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B85" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B86" t="s">
-        <v>126</v>
+        <v>187</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B87" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B88" t="s">
-        <v>76</v>
+        <v>110</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" s="1" t="s">
-        <v>14</v>
+        <v>151</v>
       </c>
       <c r="B89" t="s">
-        <v>74</v>
+        <v>170</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="B90" s="1" t="s">
-        <v>169</v>
+        <v>132</v>
+      </c>
+      <c r="B90" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>189</v>
+        <v>152</v>
+      </c>
+      <c r="B91" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" s="1" t="s">
-        <v>13</v>
+        <v>62</v>
       </c>
       <c r="B92" t="s">
-        <v>127</v>
+        <v>66</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" s="1" t="s">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="B93" t="s">
-        <v>110</v>
+        <v>64</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" s="1" t="s">
-        <v>151</v>
+        <v>2</v>
       </c>
       <c r="B94" t="s">
-        <v>170</v>
+        <v>33</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" s="1" t="s">
-        <v>132</v>
+        <v>63</v>
       </c>
       <c r="B95" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B96" t="s">
-        <v>171</v>
+        <v>36</v>
       </c>
     </row>
     <row r="97" spans="1:2">
-      <c r="A97" s="1" t="s">
-        <v>62</v>
+      <c r="A97" t="s">
+        <v>172</v>
       </c>
       <c r="B97" t="s">
-        <v>66</v>
+        <v>37</v>
       </c>
     </row>
     <row r="98" spans="1:2">
-      <c r="A98" s="1" t="s">
-        <v>64</v>
+      <c r="A98" t="s">
+        <v>173</v>
       </c>
       <c r="B98" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
     </row>
     <row r="99" spans="1:2">
-      <c r="A99" s="1" t="s">
-        <v>2</v>
+      <c r="A99" t="s">
+        <v>190</v>
       </c>
       <c r="B99" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2">
-      <c r="A100" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B100" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2">
-      <c r="A101" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="B101" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2">
-      <c r="A102" t="s">
-        <v>172</v>
-      </c>
-      <c r="B102" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2">
-      <c r="A103" t="s">
-        <v>173</v>
-      </c>
-      <c r="B103" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2">
-      <c r="A104" t="s">
-        <v>190</v>
-      </c>
-      <c r="B104" t="s">
         <v>191</v>
       </c>
     </row>
@@ -1873,10 +1833,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F34CFB7-6746-4EED-A01C-0BEF089865E6}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="48.140625" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="48.109375" customWidth="1"/>
+    <col min="2" max="2" width="29.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1975,7 +1935,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8C94458-8D2F-45A6-90CE-3561672AE312}">
   <dimension ref="A1:B89"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="79" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Fix some issues in prototype and the way it is written into master
</commit_message>
<xml_diff>
--- a/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
+++ b/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubRepos\ApsimX\Prototypes\WheatSimpleLeaf\SimpleLeafImplementation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23FC5128-BD09-426B-8BE9-80AA61BCDE75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24550676-F1E5-4E64-922C-DBF3FDF28876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{99730FEE-4914-42B9-ACDB-525A29E01521}"/>
   </bookViews>
   <sheets>
     <sheet name="SimpleLeafRenames" sheetId="1" r:id="rId1"/>
-    <sheet name="Existing Model renames" sheetId="3" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
+    <sheet name="MaxLeafSizeRenames" sheetId="4" r:id="rId2"/>
+    <sheet name="Existing Model renames" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="196">
   <si>
     <t>CohortLeaf</t>
   </si>
@@ -614,6 +615,18 @@
   </si>
   <si>
     <t>(Wheat.Leaf.Transpiration + ISoilWater.Es + MicroClimate.PrecipitationInterception)</t>
+  </si>
+  <si>
+    <t>MaxLeafSize.Script.LeafPosition</t>
+  </si>
+  <si>
+    <t>MaxLeafSize.Script.MaxLeafSize</t>
+  </si>
+  <si>
+    <t>OutputMaxLeafSize.Script.LeafPosition</t>
+  </si>
+  <si>
+    <t>OutputMaxLeafSize.Script.MaxLeafSize</t>
   </si>
 </sst>
 </file>
@@ -1026,7 +1039,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45DFA9DE-B569-4853-98A7-0B05A40C5DD2}">
-  <dimension ref="A1:B99"/>
+  <dimension ref="A1:B101"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="56.109375" customWidth="1"/>
@@ -1355,7 +1368,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="B41" t="s">
         <v>53</v>
@@ -1363,7 +1376,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="1" t="s">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="B42" t="s">
         <v>53</v>
@@ -1823,6 +1836,22 @@
       </c>
       <c r="B99" t="s">
         <v>191</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" t="s">
+        <v>192</v>
+      </c>
+      <c r="B100" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" t="s">
+        <v>193</v>
+      </c>
+      <c r="B101" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -1831,6 +1860,40 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B7E1F01-A2F7-45A9-995C-5EC6E55D65FA}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F34CFB7-6746-4EED-A01C-0BEF089865E6}">
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -1932,7 +1995,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8C94458-8D2F-45A6-90CE-3561672AE312}">
   <dimension ref="A1:B89"/>
   <sheetFormatPr defaultRowHeight="14.4"/>

</xml_diff>

<commit_message>
Bring new k and sla models to prototype
</commit_message>
<xml_diff>
--- a/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
+++ b/Prototypes/WheatSimpleLeaf/SimpleLeafImplementation/VariableRenames.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubRepos\ApsimX\Prototypes\WheatSimpleLeaf\SimpleLeafImplementation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29FB1C79-D6D1-4631-8F12-D8780C8B570D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F0F39ED-5A28-479D-8B3C-CDB4C1CDC6A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{99730FEE-4914-42B9-ACDB-525A29E01521}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="270">
   <si>
     <t>CohortLeaf</t>
   </si>
@@ -846,6 +846,9 @@
   </si>
   <si>
     <t>//[OutputMaxLeafSize].Script.LeafSize</t>
+  </si>
+  <si>
+    <t>//[Leaf].Canopy.GreenExtinctionCoefficient.VegetativePhase.FixedValue</t>
   </si>
 </sst>
 </file>
@@ -1259,7 +1262,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45DFA9DE-B569-4853-98A7-0B05A40C5DD2}">
-  <dimension ref="A1:B138"/>
+  <dimension ref="A1:B139"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="71.44140625" customWidth="1"/>
@@ -2308,65 +2311,73 @@
     </row>
     <row r="131" spans="1:2">
       <c r="A131" t="s">
-        <v>242</v>
+        <v>260</v>
       </c>
       <c r="B131" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B132" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B133" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B134" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B135" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B136" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B137" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" t="s">
+        <v>248</v>
+      </c>
+      <c r="B138" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" t="s">
         <v>258</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B139" t="s">
         <v>259</v>
       </c>
     </row>

</xml_diff>